<commit_message>
Changed modules to be a series of steps
</commit_message>
<xml_diff>
--- a/data/modules/odm_v1_to_v2/ids/odm_v1_to_v2_id_code.xlsx
+++ b/data/modules/odm_v1_to_v2/ids/odm_v1_to_v2_id_code.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/data/modules/odm_v1_to_v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9617BFE2-84EF-A94D-84C9-534410D3E708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D422652B-3BF0-2844-AACE-AF23C1AB3275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
   <sheets>
     <sheet name="id_code" sheetId="1" r:id="rId1"/>

</xml_diff>